<commit_message>
Attempting to upload without largeXGBoost file
</commit_message>
<xml_diff>
--- a/RESULTS/overall_results.xlsx
+++ b/RESULTS/overall_results.xlsx
@@ -3,24 +3,27 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="1" activeTab="4" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="pca_results" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="rf_results_transformed_data_DOSCAR_Files" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="rf_results_transformed_data_DOSCAR_Files_Initial" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="rf_results_DOSCAR_files_Initial" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="rf_results_DOSCAR_files" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="rf_results_DOSCAR_files_Initial" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="rf_results_DOSCAR_files" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="hyperparam_gridsearch_results" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Sheet2" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="rf_results_transformed_data_DOSCAR_Files" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="rf_results_transformed_data_DOSCAR_Files_Initial" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="xgb_results_transformed_data_DOSCAR_files" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -30,11 +33,13 @@
     </font>
     <font>
       <name val="Calibri"/>
-      <family val="2"/>
       <b val="1"/>
-      <color theme="1"/>
       <sz val="11"/>
-      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="11"/>
     </font>
     <font>
       <b val="1"/>
@@ -48,12 +53,27 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -81,12 +101,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
@@ -458,32 +481,32 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>dataset</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>min_energy</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>max_energy</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>energy_range</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>cum_variance</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>n_pc</t>
         </is>
@@ -644,51 +667,46 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>dataset</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>energy_range</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>cum_variance</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
-        <is>
-          <t>n_pc</t>
-        </is>
-      </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>MAE</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>MSE</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>RMSE</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="G1" s="3" t="inlineStr">
         <is>
           <t>R^2</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="H1" s="3" t="inlineStr">
         <is>
           <t>Adjusted_R^2</t>
         </is>
@@ -697,12 +715,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>DOSCAR_Files</t>
+          <t>DOSCAR_files_Initial</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>-1.46,3.27</t>
+          <t>-10.00,10.00</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -711,33 +729,30 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>2</v>
+        <v>0.1185583333333333</v>
       </c>
       <c r="E2" t="n">
-        <v>0.1788315789473685</v>
+        <v>0.02300755249999999</v>
       </c>
       <c r="F2" t="n">
-        <v>0.05429152315789479</v>
+        <v>0.1516824066924045</v>
       </c>
       <c r="G2" t="n">
-        <v>0.23300541443901</v>
+        <v>0.1073453967398629</v>
       </c>
       <c r="H2" t="n">
-        <v>-0.3100609657989537</v>
-      </c>
-      <c r="I2" t="n">
-        <v>-0.3585817423100262</v>
+        <v>1.892654603260137</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>DOSCAR_Files</t>
+          <t>DOSCAR_files_Initial</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>-1.46,3.27</t>
+          <t>-10.00,10.00</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -746,33 +761,30 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>5</v>
+        <v>0.1347083333333333</v>
       </c>
       <c r="E3" t="n">
-        <v>0.1340017543859649</v>
+        <v>0.02551839583333336</v>
       </c>
       <c r="F3" t="n">
-        <v>0.03158618649122807</v>
+        <v>0.1597447834307379</v>
       </c>
       <c r="G3" t="n">
-        <v>0.1777250305703394</v>
+        <v>0.009928869729218803</v>
       </c>
       <c r="H3" t="n">
-        <v>0.2378215313602436</v>
-      </c>
-      <c r="I3" t="n">
-        <v>0.1630981520818362</v>
+        <v>1.54453912164893</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>DOSCAR_Files</t>
+          <t>DOSCAR_files_Initial</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>-10.00,10.00</t>
+          <t>-16.14,4.12</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -781,33 +793,30 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>19</v>
+        <v>0.1496416666666666</v>
       </c>
       <c r="E4" t="n">
-        <v>0.125219298245614</v>
+        <v>0.02869168583333331</v>
       </c>
       <c r="F4" t="n">
-        <v>0.03063888087719298</v>
+        <v>0.1693862031965216</v>
       </c>
       <c r="G4" t="n">
-        <v>0.1750396551561759</v>
+        <v>-0.1131894813417751</v>
       </c>
       <c r="H4" t="n">
-        <v>0.2606801294515209</v>
-      </c>
-      <c r="I4" t="n">
-        <v>-0.1189706148841845</v>
+        <v>1.874648878197109</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>DOSCAR_Files</t>
+          <t>DOSCAR_files_Initial</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>-10.00,10.00</t>
+          <t>-16.14,4.12</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -816,28 +825,25 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>36</v>
+        <v>0.1725333333333332</v>
       </c>
       <c r="E5" t="n">
-        <v>0.1306298245614035</v>
+        <v>0.03684141166666662</v>
       </c>
       <c r="F5" t="n">
-        <v>0.03055627210526315</v>
+        <v>0.1919411672014803</v>
       </c>
       <c r="G5" t="n">
-        <v>0.1748035242930278</v>
+        <v>-0.4293852296914979</v>
       </c>
       <c r="H5" t="n">
-        <v>0.2626734890267002</v>
-      </c>
-      <c r="I5" t="n">
-        <v>-1.06451423072524</v>
+        <v>1.683619022895934</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>DOSCAR_Files</t>
+          <t>DOSCAR_files_Initial</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -851,28 +857,25 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>13</v>
+        <v>0.137975</v>
       </c>
       <c r="E6" t="n">
-        <v>0.1487280701754385</v>
+        <v>0.02963038583333332</v>
       </c>
       <c r="F6" t="n">
-        <v>0.04016805105263157</v>
+        <v>0.1721347897240221</v>
       </c>
       <c r="G6" t="n">
-        <v>0.2004196872880296</v>
+        <v>-0.14960947325879</v>
       </c>
       <c r="H6" t="n">
-        <v>0.03074011014148359</v>
-      </c>
-      <c r="I6" t="n">
-        <v>-0.2622919495831841</v>
+        <v>3.529140841169338</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>DOSCAR_Files</t>
+          <t>DOSCAR_files_Initial</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -886,22 +889,19 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>23</v>
+        <v>0.1534166666666666</v>
       </c>
       <c r="E7" t="n">
-        <v>0.1526263157894737</v>
+        <v>0.03513465333333331</v>
       </c>
       <c r="F7" t="n">
-        <v>0.03828791175438596</v>
+        <v>0.1874424000415416</v>
       </c>
       <c r="G7" t="n">
-        <v>0.1956729714456904</v>
+        <v>-0.3631658574700249</v>
       </c>
       <c r="H7" t="n">
-        <v>0.07610809692153486</v>
-      </c>
-      <c r="I7" t="n">
-        <v>-0.5678165627998197</v>
+        <v>2.363165857470025</v>
       </c>
     </row>
   </sheetData>
@@ -915,51 +915,46 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>dataset</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>energy_range</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>cum_variance</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
-        <is>
-          <t>n_pc</t>
-        </is>
-      </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>MAE</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>MSE</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>RMSE</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="G1" s="3" t="inlineStr">
         <is>
           <t>R^2</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="H1" s="3" t="inlineStr">
         <is>
           <t>Adjusted_R^2</t>
         </is>
@@ -968,12 +963,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>DOSCAR_Files_Initial</t>
+          <t>DOSCAR_files</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>-10.00,10.00</t>
+          <t>-1.46,3.27</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -982,33 +977,30 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>22</v>
+        <v>0.1788315789473685</v>
       </c>
       <c r="E2" t="n">
-        <v>0.1208333333333333</v>
+        <v>0.05429152315789479</v>
       </c>
       <c r="F2" t="n">
-        <v>0.02383059166666667</v>
+        <v>0.23300541443901</v>
       </c>
       <c r="G2" t="n">
-        <v>0.1543716025267169</v>
+        <v>-0.3100609657989537</v>
       </c>
       <c r="H2" t="n">
-        <v>0.0754128519466517</v>
-      </c>
-      <c r="I2" t="n">
-        <v>1.924587148053348</v>
+        <v>-0.3585817423100262</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>DOSCAR_Files_Initial</t>
+          <t>DOSCAR_files</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>-10.00,10.00</t>
+          <t>-1.46,3.27</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1017,33 +1009,30 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>31</v>
+        <v>0.1340017543859649</v>
       </c>
       <c r="E3" t="n">
-        <v>0.1344416666666667</v>
+        <v>0.03158618649122807</v>
       </c>
       <c r="F3" t="n">
-        <v>0.0254661941666667</v>
+        <v>0.1777250305703394</v>
       </c>
       <c r="G3" t="n">
-        <v>0.1595813089514768</v>
+        <v>0.2378215313602436</v>
       </c>
       <c r="H3" t="n">
-        <v>0.01195420719385554</v>
-      </c>
-      <c r="I3" t="n">
-        <v>1.543425186043379</v>
+        <v>0.1630981520818362</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>DOSCAR_Files_Initial</t>
+          <t>DOSCAR_files</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>-16.14,4.12</t>
+          <t>-10.00,10.00</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -1052,33 +1041,30 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>25</v>
+        <v>0.1319859649122807</v>
       </c>
       <c r="E4" t="n">
-        <v>0.1555916666666666</v>
+        <v>0.03337958421052633</v>
       </c>
       <c r="F4" t="n">
-        <v>0.0297696708333333</v>
+        <v>0.18270080517208</v>
       </c>
       <c r="G4" t="n">
-        <v>0.1725388965808385</v>
+        <v>0.1945466292844145</v>
       </c>
       <c r="H4" t="n">
-        <v>-0.1550134985854765</v>
-      </c>
-      <c r="I4" t="n">
-        <v>1.907510606031446</v>
+        <v>-0.2190645610830484</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>DOSCAR_Files_Initial</t>
+          <t>DOSCAR_files</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>-16.14,4.12</t>
+          <t>-10.00,10.00</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -1087,28 +1073,25 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>34</v>
+        <v>0.1310824561403509</v>
       </c>
       <c r="E5" t="n">
-        <v>0.1741749999999999</v>
+        <v>0.03069698333333332</v>
       </c>
       <c r="F5" t="n">
-        <v>0.0368889258333333</v>
+        <v>0.1752055459548393</v>
       </c>
       <c r="G5" t="n">
-        <v>0.1920649000555107</v>
+        <v>0.2592781102157529</v>
       </c>
       <c r="H5" t="n">
-        <v>-0.4312286999865274</v>
-      </c>
-      <c r="I5" t="n">
-        <v>1.684500682602252</v>
+        <v>-1.074021291395892</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>DOSCAR_Files_Initial</t>
+          <t>DOSCAR_files</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1122,28 +1105,25 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>16</v>
+        <v>0.1483789473684211</v>
       </c>
       <c r="E6" t="n">
-        <v>0.1393333333333332</v>
+        <v>0.03958468491228069</v>
       </c>
       <c r="F6" t="n">
-        <v>0.03040609333333331</v>
+        <v>0.1989590030943076</v>
       </c>
       <c r="G6" t="n">
-        <v>0.1743734306978368</v>
+        <v>0.04481680508002561</v>
       </c>
       <c r="H6" t="n">
-        <v>-0.1797056284521077</v>
-      </c>
-      <c r="I6" t="n">
-        <v>3.595352382594637</v>
+        <v>-0.2439595096632226</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>DOSCAR_Files_Initial</t>
+          <t>DOSCAR_files</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1157,22 +1137,19 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>22</v>
+        <v>0.152878947368421</v>
       </c>
       <c r="E7" t="n">
-        <v>0.1518916666666666</v>
+        <v>0.03832600192982456</v>
       </c>
       <c r="F7" t="n">
-        <v>0.03422941249999997</v>
+        <v>0.1957702784638786</v>
       </c>
       <c r="G7" t="n">
-        <v>0.1850119252913173</v>
+        <v>0.07518897641947375</v>
       </c>
       <c r="H7" t="n">
-        <v>-0.3280440253266868</v>
-      </c>
-      <c r="I7" t="n">
-        <v>2.328044025326687</v>
+        <v>-0.5693762824396809</v>
       </c>
     </row>
   </sheetData>
@@ -1186,8 +1163,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:H7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
@@ -1207,30 +1184,25 @@
       </c>
       <c r="D1" s="2" t="inlineStr">
         <is>
-          <t>n_pc</t>
+          <t>MAE</t>
         </is>
       </c>
       <c r="E1" s="2" t="inlineStr">
         <is>
-          <t>MAE</t>
+          <t>MSE</t>
         </is>
       </c>
       <c r="F1" s="2" t="inlineStr">
         <is>
-          <t>MSE</t>
+          <t>RMSE</t>
         </is>
       </c>
       <c r="G1" s="2" t="inlineStr">
         <is>
-          <t>RMSE</t>
+          <t>R^2</t>
         </is>
       </c>
       <c r="H1" s="2" t="inlineStr">
-        <is>
-          <t>R^2</t>
-        </is>
-      </c>
-      <c r="I1" s="2" t="inlineStr">
         <is>
           <t>Adjusted_R^2</t>
         </is>
@@ -1239,12 +1211,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>DOSCAR_files_Initial</t>
+          <t>DOSCAR_Files</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>-10.00,10.00</t>
+          <t>-1.46,3.27</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -1253,33 +1225,30 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>22</v>
+        <v>0.1562341435693673</v>
       </c>
       <c r="E2" t="n">
-        <v>0.1208333333333333</v>
+        <v>0.04128177322297947</v>
       </c>
       <c r="F2" t="n">
-        <v>0.02383059166666667</v>
+        <v>0.2031791653270076</v>
       </c>
       <c r="G2" t="n">
-        <v>0.1543716025267169</v>
+        <v>0.003865860585537728</v>
       </c>
       <c r="H2" t="n">
-        <v>0.0754128519466517</v>
-      </c>
-      <c r="I2" t="n">
-        <v>1.924587148053348</v>
+        <v>-0.0330279964298128</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>DOSCAR_files_Initial</t>
+          <t>DOSCAR_Files</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>-10.00,10.00</t>
+          <t>-1.46,3.27</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1288,33 +1257,30 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>31</v>
+        <v>0.1359383221943748</v>
       </c>
       <c r="E3" t="n">
-        <v>0.1344416666666667</v>
+        <v>0.03078673395670935</v>
       </c>
       <c r="F3" t="n">
-        <v>0.0254661941666667</v>
+        <v>0.1754614885287064</v>
       </c>
       <c r="G3" t="n">
-        <v>0.1595813089514768</v>
+        <v>0.2571124169085471</v>
       </c>
       <c r="H3" t="n">
-        <v>0.01195420719385554</v>
-      </c>
-      <c r="I3" t="n">
-        <v>1.543425186043379</v>
+        <v>0.184280300919189</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>DOSCAR_files_Initial</t>
+          <t>DOSCAR_Files</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>-16.14,4.12</t>
+          <t>-10.00,10.00</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -1323,33 +1289,30 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>25</v>
+        <v>0.1296212306052505</v>
       </c>
       <c r="E4" t="n">
-        <v>0.1555916666666666</v>
+        <v>0.031997332320077</v>
       </c>
       <c r="F4" t="n">
-        <v>0.0297696708333333</v>
+        <v>0.1788779816525136</v>
       </c>
       <c r="G4" t="n">
-        <v>0.1725388965808385</v>
+        <v>0.2279005331952159</v>
       </c>
       <c r="H4" t="n">
-        <v>-0.1550134985854765</v>
-      </c>
-      <c r="I4" t="n">
-        <v>1.907510606031446</v>
+        <v>-0.1685829767856193</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>DOSCAR_files_Initial</t>
+          <t>DOSCAR_Files</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>-16.14,4.12</t>
+          <t>-10.00,10.00</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -1358,28 +1321,25 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>34</v>
+        <v>0.1420304093567251</v>
       </c>
       <c r="E5" t="n">
-        <v>0.1741749999999999</v>
+        <v>0.03597623906432748</v>
       </c>
       <c r="F5" t="n">
-        <v>0.0368889258333333</v>
+        <v>0.1896740337113319</v>
       </c>
       <c r="G5" t="n">
-        <v>0.1920649000555107</v>
+        <v>0.1318890362063205</v>
       </c>
       <c r="H5" t="n">
-        <v>-0.4312286999865274</v>
-      </c>
-      <c r="I5" t="n">
-        <v>1.684500682602252</v>
+        <v>-1.430710698622303</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>DOSCAR_files_Initial</t>
+          <t>DOSCAR_Files</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1393,28 +1353,25 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>16</v>
+        <v>0.1481298405282304</v>
       </c>
       <c r="E6" t="n">
-        <v>0.1393333333333332</v>
+        <v>0.03740489726623729</v>
       </c>
       <c r="F6" t="n">
-        <v>0.03040609333333331</v>
+        <v>0.1934034572241078</v>
       </c>
       <c r="G6" t="n">
-        <v>0.1743734306978368</v>
+        <v>0.09741534243377081</v>
       </c>
       <c r="H6" t="n">
-        <v>-0.1797056284521077</v>
-      </c>
-      <c r="I6" t="n">
-        <v>3.595352382594637</v>
+        <v>-0.1754590889234613</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>DOSCAR_files_Initial</t>
+          <t>DOSCAR_Files</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1428,22 +1385,19 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>22</v>
+        <v>0.151490834536509</v>
       </c>
       <c r="E7" t="n">
-        <v>0.1518916666666666</v>
+        <v>0.04073658745354566</v>
       </c>
       <c r="F7" t="n">
-        <v>0.03422941249999997</v>
+        <v>0.2018330682855158</v>
       </c>
       <c r="G7" t="n">
-        <v>0.1850119252913173</v>
+        <v>0.01702125859430481</v>
       </c>
       <c r="H7" t="n">
-        <v>-0.3280440253266868</v>
-      </c>
-      <c r="I7" t="n">
-        <v>2.328044025326687</v>
+        <v>-0.6680851369308767</v>
       </c>
     </row>
   </sheetData>
@@ -1457,51 +1411,535 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:H17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <cols>
+    <col width="12.109375" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="12.5546875" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="12.77734375" bestFit="1" customWidth="1" min="3" max="3"/>
+    <col width="12" bestFit="1" customWidth="1" min="4" max="6"/>
+    <col width="12.6640625" bestFit="1" customWidth="1" min="7" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>energy_range</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>cum_variance</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>MAE</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>MSE</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>RMSE</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>R^2</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>Adjusted_R^2</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>DOSCAR_files</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>-1.46,3.27</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>0.80</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>0.1788315789473685</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.05429152315789479</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.23300541443901</v>
+      </c>
+      <c r="G2" t="n">
+        <v>-0.3100609657989537</v>
+      </c>
+      <c r="H2" t="n">
+        <v>-0.3585817423100262</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>DOSCAR_files</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>-1.46,3.27</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>0.90</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>0.1340017543859649</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.03158618649122807</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.1777250305703394</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0.2378215313602436</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.1630981520818362</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>DOSCAR_files</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>-10.00,10.00</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>0.80</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>0.125219298245614</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.03063888087719298</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.1750396551561759</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.2606801294515209</v>
+      </c>
+      <c r="H4" t="n">
+        <v>-0.1189706148841845</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>DOSCAR_files</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>-10.00,10.00</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>0.90</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>0.1306298245614035</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.03055627210526315</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.1748035242930278</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0.2626734890267002</v>
+      </c>
+      <c r="H5" t="n">
+        <v>-1.06451423072524</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>DOSCAR_files</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>-5.00,5.00</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>0.80</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>0.1487280701754385</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.04016805105263157</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.2004196872880296</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.03074011014148359</v>
+      </c>
+      <c r="H6" t="n">
+        <v>-0.2622919495831841</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>DOSCAR_files</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>-5.00,5.00</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>0.90</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>0.1526263157894737</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.03828791175438596</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.1956729714456904</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0.07610809692153486</v>
+      </c>
+      <c r="H7" t="n">
+        <v>-0.5678165627998197</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>energy_range</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>cum_variance</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>MAE</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>MSE</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>RMSE</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>R^2</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>Adjusted_R^2</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>DOSCAR_Files</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>-1.46,3.27</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>0.80</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>0.1562341435693673</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0.04128177322297947</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0.2031791653270076</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0.003865860585537728</v>
+      </c>
+      <c r="H12" t="n">
+        <v>-0.0330279964298128</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>DOSCAR_Files</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>-1.46,3.27</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>0.90</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>0.1359383221943748</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0.03078673395670935</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0.1754614885287064</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0.2571124169085471</v>
+      </c>
+      <c r="H13" t="n">
+        <v>0.184280300919189</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>DOSCAR_Files</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>-10.00,10.00</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>0.80</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>0.1296212306052505</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0.031997332320077</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0.1788779816525136</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0.2279005331952159</v>
+      </c>
+      <c r="H14" t="n">
+        <v>-0.1685829767856193</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>DOSCAR_Files</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>-10.00,10.00</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>0.90</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>0.1420304093567251</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0.03597623906432748</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0.1896740337113319</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0.1318890362063205</v>
+      </c>
+      <c r="H15" t="n">
+        <v>-1.430710698622303</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>DOSCAR_Files</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>-5.00,5.00</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>0.80</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>0.1481298405282304</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0.03740489726623729</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0.1934034572241078</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0.09741534243377081</v>
+      </c>
+      <c r="H16" t="n">
+        <v>-0.1754590889234613</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>DOSCAR_Files</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>-5.00,5.00</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>0.90</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>0.151490834536509</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0.04073658745354566</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0.2018330682855158</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0.01702125859430481</v>
+      </c>
+      <c r="H17" t="n">
+        <v>-0.6680851369308767</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>dataset</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>energy_range</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>cum_variance</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
-        <is>
-          <t>n_pc</t>
-        </is>
-      </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>MAE</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>MSE</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>RMSE</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="G1" s="3" t="inlineStr">
         <is>
           <t>R^2</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="H1" s="3" t="inlineStr">
         <is>
           <t>Adjusted_R^2</t>
         </is>
@@ -1510,7 +1948,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>DOSCAR_files</t>
+          <t>DOSCAR_Files</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1524,28 +1962,25 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>2</v>
+        <v>0.1788315789473685</v>
       </c>
       <c r="E2" t="n">
-        <v>0.1788315789473685</v>
+        <v>0.05429152315789479</v>
       </c>
       <c r="F2" t="n">
-        <v>0.05429152315789479</v>
+        <v>0.23300541443901</v>
       </c>
       <c r="G2" t="n">
-        <v>0.23300541443901</v>
+        <v>-0.3100609657989537</v>
       </c>
       <c r="H2" t="n">
-        <v>-0.3100609657989537</v>
-      </c>
-      <c r="I2" t="n">
         <v>-0.3585817423100262</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>DOSCAR_files</t>
+          <t>DOSCAR_Files</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1559,28 +1994,25 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>5</v>
+        <v>0.1340017543859649</v>
       </c>
       <c r="E3" t="n">
-        <v>0.1340017543859649</v>
+        <v>0.03158618649122807</v>
       </c>
       <c r="F3" t="n">
-        <v>0.03158618649122807</v>
+        <v>0.1777250305703394</v>
       </c>
       <c r="G3" t="n">
-        <v>0.1777250305703394</v>
+        <v>0.2378215313602436</v>
       </c>
       <c r="H3" t="n">
-        <v>0.2378215313602436</v>
-      </c>
-      <c r="I3" t="n">
         <v>0.1630981520818362</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>DOSCAR_files</t>
+          <t>DOSCAR_Files</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1594,28 +2026,25 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>19</v>
+        <v>0.1319859649122807</v>
       </c>
       <c r="E4" t="n">
-        <v>0.125219298245614</v>
+        <v>0.03337958421052633</v>
       </c>
       <c r="F4" t="n">
-        <v>0.03063888087719298</v>
+        <v>0.18270080517208</v>
       </c>
       <c r="G4" t="n">
-        <v>0.1750396551561759</v>
+        <v>0.1945466292844145</v>
       </c>
       <c r="H4" t="n">
-        <v>0.2606801294515209</v>
-      </c>
-      <c r="I4" t="n">
-        <v>-0.1189706148841845</v>
+        <v>-0.2190645610830484</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>DOSCAR_files</t>
+          <t>DOSCAR_Files</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1629,28 +2058,25 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>36</v>
+        <v>0.1310824561403509</v>
       </c>
       <c r="E5" t="n">
-        <v>0.1306298245614035</v>
+        <v>0.03069698333333332</v>
       </c>
       <c r="F5" t="n">
-        <v>0.03055627210526315</v>
+        <v>0.1752055459548393</v>
       </c>
       <c r="G5" t="n">
-        <v>0.1748035242930278</v>
+        <v>0.2592781102157529</v>
       </c>
       <c r="H5" t="n">
-        <v>0.2626734890267002</v>
-      </c>
-      <c r="I5" t="n">
-        <v>-1.06451423072524</v>
+        <v>-1.074021291395892</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>DOSCAR_files</t>
+          <t>DOSCAR_Files</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1664,30 +2090,523 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>13</v>
+        <v>0.1483789473684211</v>
       </c>
       <c r="E6" t="n">
-        <v>0.1487280701754385</v>
+        <v>0.03958468491228069</v>
       </c>
       <c r="F6" t="n">
-        <v>0.04016805105263157</v>
+        <v>0.1989590030943076</v>
       </c>
       <c r="G6" t="n">
-        <v>0.2004196872880296</v>
+        <v>0.04481680508002561</v>
       </c>
       <c r="H6" t="n">
-        <v>0.03074011014148359</v>
-      </c>
-      <c r="I6" t="n">
-        <v>-0.2622919495831841</v>
+        <v>-0.2439595096632226</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>DOSCAR_Files</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>-5.00,5.00</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>0.90</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>0.152878947368421</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.03832600192982456</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.1957702784638786</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0.07518897641947375</v>
+      </c>
+      <c r="H7" t="n">
+        <v>-0.5693762824396809</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>energy_range</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>cum_variance</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>MAE</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>MSE</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>RMSE</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>R^2</t>
+        </is>
+      </c>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>Adjusted_R^2</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>DOSCAR_Files_Initial</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>-10.00,10.00</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>0.80</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>0.1185583333333333</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.02300755249999999</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.1516824066924045</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0.1073453967398629</v>
+      </c>
+      <c r="H2" t="n">
+        <v>1.892654603260137</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>DOSCAR_Files_Initial</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>-10.00,10.00</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>0.90</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>0.1347083333333333</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.02551839583333336</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.1597447834307379</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0.009928869729218803</v>
+      </c>
+      <c r="H3" t="n">
+        <v>1.54453912164893</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>DOSCAR_Files_Initial</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>-16.14,4.12</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>0.80</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>0.1496416666666666</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.02869168583333331</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.1693862031965216</v>
+      </c>
+      <c r="G4" t="n">
+        <v>-0.1131894813417751</v>
+      </c>
+      <c r="H4" t="n">
+        <v>1.874648878197109</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>DOSCAR_Files_Initial</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>-16.14,4.12</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>0.90</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>0.1725333333333332</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.03684141166666662</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.1919411672014803</v>
+      </c>
+      <c r="G5" t="n">
+        <v>-0.4293852296914979</v>
+      </c>
+      <c r="H5" t="n">
+        <v>1.683619022895934</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>DOSCAR_Files_Initial</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>-5.00,5.00</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>0.80</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>0.137975</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.02963038583333332</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.1721347897240221</v>
+      </c>
+      <c r="G6" t="n">
+        <v>-0.14960947325879</v>
+      </c>
+      <c r="H6" t="n">
+        <v>3.529140841169338</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>DOSCAR_Files_Initial</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>-5.00,5.00</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>0.90</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>0.1534166666666666</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.03513465333333331</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.1874424000415416</v>
+      </c>
+      <c r="G7" t="n">
+        <v>-0.3631658574700249</v>
+      </c>
+      <c r="H7" t="n">
+        <v>2.363165857470025</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>energy_range</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>cum_variance</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>MAE</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>MSE</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>RMSE</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>R^2</t>
+        </is>
+      </c>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>Adjusted_R^2</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
           <t>DOSCAR_files</t>
         </is>
       </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>-1.46,3.27</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>0.80</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>0.2080599773557562</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.09679153302620662</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.3111133764822828</v>
+      </c>
+      <c r="G2" t="n">
+        <v>-1.33559130158673</v>
+      </c>
+      <c r="H2" t="n">
+        <v>-1.422094683126979</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>DOSCAR_files</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>-1.46,3.27</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>0.90</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>0.160469670138861</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.04495700089404833</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.2120306602688591</v>
+      </c>
+      <c r="G3" t="n">
+        <v>-0.08481782394268644</v>
+      </c>
+      <c r="H3" t="n">
+        <v>-0.1911725125645185</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>DOSCAR_files</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>-10.00,10.00</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>0.80</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>0.1281089411806642</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.0292253935525506</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.1709543610223226</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.2947877481359361</v>
+      </c>
+      <c r="H4" t="n">
+        <v>-0.067348273091556</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>DOSCAR_files</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>-10.00,10.00</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>0.90</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>0.127242969253607</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.0275487526003409</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.165978169047441</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0.3352452954175235</v>
+      </c>
+      <c r="H5" t="n">
+        <v>-0.8613131728309344</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>DOSCAR_files</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>-5.00,5.00</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>0.80</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>0.149748526518805</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.04115635235899723</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.2028702845638001</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.006892281077039875</v>
+      </c>
+      <c r="H6" t="n">
+        <v>-0.2933495874345526</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>DOSCAR_files</t>
+        </is>
+      </c>
       <c r="B7" t="inlineStr">
         <is>
           <t>-5.00,5.00</t>
@@ -1699,22 +2618,19 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>23</v>
+        <v>0.1630195843546014</v>
       </c>
       <c r="E7" t="n">
-        <v>0.1526263157894737</v>
+        <v>0.04607930403670059</v>
       </c>
       <c r="F7" t="n">
-        <v>0.03828791175438596</v>
+        <v>0.2146609047700596</v>
       </c>
       <c r="G7" t="n">
-        <v>0.1956729714456904</v>
+        <v>-0.1118991333895814</v>
       </c>
       <c r="H7" t="n">
-        <v>0.07610809692153486</v>
-      </c>
-      <c r="I7" t="n">
-        <v>-0.5678165627998197</v>
+        <v>-0.8868591354489865</v>
       </c>
     </row>
   </sheetData>

</xml_diff>